<commit_message>
Make the updated Claim Status and Notes cells easy to find
The Notes column (AB) is the last of 28 columns and only 47 of 1086 rows
are populated, with the first at row 151, so the column reads as empty
when scrolling from the top.

Widen Notes from 12 to 70 characters and shade the Claim Status and
Notes cells of the 47 updated rows so they stand out. Cell values are
unchanged.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012tS5RtxREUtPc7HhmELBS5
</commit_message>
<xml_diff>
--- a/Specialty Claims Pending 2026-S1.xlsx
+++ b/Specialty Claims Pending 2026-S1.xlsx
@@ -33,7 +33,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -50,6 +50,11 @@
         <fgColor rgb="FF7F6000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -63,13 +68,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -458,7 +467,7 @@
     <col width="22" customWidth="1" min="25" max="25"/>
     <col width="19" customWidth="1" min="26" max="26"/>
     <col width="24" customWidth="1" min="27" max="27"/>
-    <col width="12" customWidth="1" min="28" max="28"/>
+    <col width="70" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -14892,7 +14901,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J151" t="inlineStr">
+      <c r="J151" s="3" t="inlineStr">
         <is>
           <t>Finalized</t>
         </is>
@@ -14945,7 +14954,7 @@
       <c r="AA151" t="n">
         <v>116</v>
       </c>
-      <c r="AB151" t="inlineStr">
+      <c r="AB151" s="4" t="inlineStr">
         <is>
           <t>Adjusted - CPT 93923 bundles with 93925 and 93970 - 93923 billed on claim 568254615</t>
         </is>
@@ -19704,7 +19713,7 @@
           <t>UnitedHealthcare Community Plan / Arizona Long Term Care</t>
         </is>
       </c>
-      <c r="J201" t="inlineStr">
+      <c r="J201" s="3" t="inlineStr">
         <is>
           <t>Denied</t>
         </is>
@@ -19757,7 +19766,7 @@
       <c r="AA201" t="n">
         <v>80</v>
       </c>
-      <c r="AB201" t="inlineStr">
+      <c r="AB201" s="4" t="inlineStr">
         <is>
           <t>Corrected service line 1 - Changed to 99492, and resubmitted - Processed date 06/10/2026</t>
         </is>
@@ -20551,7 +20560,7 @@
           <t>Molina Complete Care of Arizona (Magellan Complete Care AZ)</t>
         </is>
       </c>
-      <c r="J210" t="inlineStr">
+      <c r="J210" s="3" t="inlineStr">
         <is>
           <t>Finalized</t>
         </is>
@@ -20609,7 +20618,7 @@
       <c r="AA210" t="n">
         <v>79</v>
       </c>
-      <c r="AB210" t="inlineStr">
+      <c r="AB210" s="4" t="inlineStr">
         <is>
           <t>Billed PT according to ABN charges agreed.</t>
         </is>
@@ -21104,7 +21113,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J216" t="inlineStr">
+      <c r="J216" s="3" t="inlineStr">
         <is>
           <t>Denied</t>
         </is>
@@ -21157,7 +21166,7 @@
       <c r="AA216" t="n">
         <v>88</v>
       </c>
-      <c r="AB216" t="inlineStr">
+      <c r="AB216" s="4" t="inlineStr">
         <is>
           <t>DMinker30A corrected claim and resubmitted</t>
         </is>
@@ -21202,7 +21211,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J217" t="inlineStr">
+      <c r="J217" s="3" t="inlineStr">
         <is>
           <t>Denied</t>
         </is>
@@ -21255,7 +21264,7 @@
       <c r="AA217" t="n">
         <v>88</v>
       </c>
-      <c r="AB217" t="inlineStr">
+      <c r="AB217" s="4" t="inlineStr">
         <is>
           <t>DMinker30A corrected claim and resubmitted</t>
         </is>
@@ -29442,7 +29451,7 @@
           <t>Arizona Complete Health (Centene)</t>
         </is>
       </c>
-      <c r="J308" t="inlineStr">
+      <c r="J308" s="3" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -29485,7 +29494,7 @@
       <c r="AA308" t="n">
         <v>89</v>
       </c>
-      <c r="AB308" t="inlineStr">
+      <c r="AB308" s="4" t="inlineStr">
         <is>
           <t>On hold - Missing MR - Uploaded MR on portal</t>
         </is>
@@ -35446,7 +35455,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J373" t="inlineStr">
+      <c r="J373" s="3" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
@@ -35509,7 +35518,7 @@
       <c r="AA373" t="n">
         <v>87</v>
       </c>
-      <c r="AB373" t="inlineStr">
+      <c r="AB373" s="4" t="inlineStr">
         <is>
           <t>Removed 20936, and resubmited</t>
         </is>
@@ -36276,7 +36285,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J383" t="inlineStr">
+      <c r="J383" s="3" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -36319,7 +36328,7 @@
       <c r="AA383" t="n">
         <v>79</v>
       </c>
-      <c r="AB383" t="inlineStr">
+      <c r="AB383" s="4" t="inlineStr">
         <is>
           <t>Waiting for Juan to send the ultrasounds to me</t>
         </is>
@@ -36364,7 +36373,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J384" t="inlineStr">
+      <c r="J384" s="3" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -36407,7 +36416,7 @@
       <c r="AA384" t="n">
         <v>79</v>
       </c>
-      <c r="AB384" t="inlineStr">
+      <c r="AB384" s="4" t="inlineStr">
         <is>
           <t>Waiting for Juan to send the ultrasounds to me</t>
         </is>
@@ -36452,7 +36461,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J385" t="inlineStr">
+      <c r="J385" s="3" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -36495,7 +36504,7 @@
       <c r="AA385" t="n">
         <v>79</v>
       </c>
-      <c r="AB385" t="inlineStr">
+      <c r="AB385" s="4" t="inlineStr">
         <is>
           <t>Waiting for Juan to send the ultrasounds to me</t>
         </is>
@@ -37201,7 +37210,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J393" t="inlineStr">
+      <c r="J393" s="3" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
@@ -37259,7 +37268,7 @@
       <c r="AA393" t="n">
         <v>87</v>
       </c>
-      <c r="AB393" t="inlineStr">
+      <c r="AB393" s="4" t="inlineStr">
         <is>
           <t>Removed 20936, and resubmited</t>
         </is>
@@ -37304,7 +37313,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J394" t="inlineStr">
+      <c r="J394" s="3" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
@@ -37362,7 +37371,7 @@
       <c r="AA394" t="n">
         <v>87</v>
       </c>
-      <c r="AB394" t="inlineStr">
+      <c r="AB394" s="4" t="inlineStr">
         <is>
           <t>Removed 20936, and resubmited</t>
         </is>
@@ -37407,7 +37416,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J395" t="inlineStr">
+      <c r="J395" s="3" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
@@ -37470,7 +37479,7 @@
       <c r="AA395" t="n">
         <v>87</v>
       </c>
-      <c r="AB395" t="inlineStr">
+      <c r="AB395" s="4" t="inlineStr">
         <is>
           <t>Removed 20936, and resubmited</t>
         </is>
@@ -52086,7 +52095,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J556" t="inlineStr">
+      <c r="J556" s="3" t="inlineStr">
         <is>
           <t>Denied</t>
         </is>
@@ -52144,7 +52153,7 @@
       <c r="AA556" t="n">
         <v>87</v>
       </c>
-      <c r="AB556" t="inlineStr">
+      <c r="AB556" s="4" t="inlineStr">
         <is>
           <t>Uploaded MR - PIQ-88944138 - Processed Date 05/28/2026</t>
         </is>
@@ -52189,7 +52198,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J557" t="inlineStr">
+      <c r="J557" s="3" t="inlineStr">
         <is>
           <t>Denied</t>
         </is>
@@ -52247,7 +52256,7 @@
       <c r="AA557" t="n">
         <v>87</v>
       </c>
-      <c r="AB557" t="inlineStr">
+      <c r="AB557" s="4" t="inlineStr">
         <is>
           <t>Uploaded MR - PIQ-88944138 - Processed Date 05/28/2026</t>
         </is>
@@ -52292,7 +52301,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J558" t="inlineStr">
+      <c r="J558" s="3" t="inlineStr">
         <is>
           <t>Denied</t>
         </is>
@@ -52350,7 +52359,7 @@
       <c r="AA558" t="n">
         <v>87</v>
       </c>
-      <c r="AB558" t="inlineStr">
+      <c r="AB558" s="4" t="inlineStr">
         <is>
           <t>Uploaded MR - PIQ-88944138 - Processed Date 05/28/2026</t>
         </is>
@@ -54042,7 +54051,7 @@
           <t>Mercy Care RBHA</t>
         </is>
       </c>
-      <c r="J578" t="inlineStr">
+      <c r="J578" s="3" t="inlineStr">
         <is>
           <t>Denied</t>
         </is>
@@ -54095,7 +54104,7 @@
       <c r="AA578" t="n">
         <v>78</v>
       </c>
-      <c r="AB578" t="inlineStr">
+      <c r="AB578" s="4" t="inlineStr">
         <is>
           <t>UHC not active on DOS - Resubmitted to Mercy Care (secondary) - Processed date 06/10/2026</t>
         </is>
@@ -54140,7 +54149,7 @@
           <t>Mercy Care RBHA</t>
         </is>
       </c>
-      <c r="J579" t="inlineStr">
+      <c r="J579" s="3" t="inlineStr">
         <is>
           <t>Denied</t>
         </is>
@@ -54193,7 +54202,7 @@
       <c r="AA579" t="n">
         <v>78</v>
       </c>
-      <c r="AB579" t="inlineStr">
+      <c r="AB579" s="4" t="inlineStr">
         <is>
           <t>UHC not active on DOS - Resubmitted to Mercy Care (secondary) - Processed date 06/10/2026</t>
         </is>
@@ -54238,7 +54247,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J580" t="inlineStr">
+      <c r="J580" s="3" t="inlineStr">
         <is>
           <t>Denied</t>
         </is>
@@ -54301,7 +54310,7 @@
       <c r="AA580" t="n">
         <v>79</v>
       </c>
-      <c r="AB580" t="inlineStr">
+      <c r="AB580" s="4" t="inlineStr">
         <is>
           <t>Uploaded MR - PIQ-88975230 - Processed date 08/08/2026</t>
         </is>
@@ -54718,7 +54727,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J585" t="inlineStr">
+      <c r="J585" s="3" t="inlineStr">
         <is>
           <t>PAID</t>
         </is>
@@ -54771,7 +54780,7 @@
       <c r="AA585" t="n">
         <v>79</v>
       </c>
-      <c r="AB585" t="inlineStr">
+      <c r="AB585" s="4" t="inlineStr">
         <is>
           <t>Pending posting</t>
         </is>
@@ -54816,7 +54825,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J586" t="inlineStr">
+      <c r="J586" s="3" t="inlineStr">
         <is>
           <t>PAID</t>
         </is>
@@ -54869,7 +54878,7 @@
       <c r="AA586" t="n">
         <v>79</v>
       </c>
-      <c r="AB586" t="inlineStr">
+      <c r="AB586" s="4" t="inlineStr">
         <is>
           <t>Pending posting</t>
         </is>
@@ -54914,7 +54923,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J587" t="inlineStr">
+      <c r="J587" s="3" t="inlineStr">
         <is>
           <t>PAID</t>
         </is>
@@ -54967,7 +54976,7 @@
       <c r="AA587" t="n">
         <v>79</v>
       </c>
-      <c r="AB587" t="inlineStr">
+      <c r="AB587" s="4" t="inlineStr">
         <is>
           <t>Pending posting</t>
         </is>
@@ -63309,7 +63318,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J682" t="inlineStr">
+      <c r="J682" s="3" t="inlineStr">
         <is>
           <t>Denied</t>
         </is>
@@ -63362,7 +63371,7 @@
       <c r="AA682" t="n">
         <v>82</v>
       </c>
-      <c r="AB682" t="inlineStr">
+      <c r="AB682" s="4" t="inlineStr">
         <is>
           <t>Checking with auth team</t>
         </is>
@@ -64938,7 +64947,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J700" t="inlineStr">
+      <c r="J700" s="3" t="inlineStr">
         <is>
           <t>Denied</t>
         </is>
@@ -64986,7 +64995,7 @@
       <c r="AA700" t="n">
         <v>86</v>
       </c>
-      <c r="AB700" t="inlineStr">
+      <c r="AB700" s="4" t="inlineStr">
         <is>
           <t>Resubmitted with 63030+63035</t>
         </is>
@@ -65031,7 +65040,7 @@
           <t>LIEN 03</t>
         </is>
       </c>
-      <c r="J701" t="inlineStr">
+      <c r="J701" s="3" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
@@ -65094,7 +65103,7 @@
       <c r="AA701" t="n">
         <v>85</v>
       </c>
-      <c r="AB701" t="inlineStr">
+      <c r="AB701" s="4" t="inlineStr">
         <is>
           <t>Remove CPT A6219, and resubmitted</t>
         </is>
@@ -67150,7 +67159,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J724" t="inlineStr">
+      <c r="J724" s="3" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
@@ -67203,7 +67212,7 @@
       <c r="AA724" t="n">
         <v>82</v>
       </c>
-      <c r="AB724" t="inlineStr">
+      <c r="AB724" s="4" t="inlineStr">
         <is>
           <t>Waiting for Bri's reply on how to get WCEOB</t>
         </is>
@@ -67248,7 +67257,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J725" t="inlineStr">
+      <c r="J725" s="3" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
@@ -67301,7 +67310,7 @@
       <c r="AA725" t="n">
         <v>82</v>
       </c>
-      <c r="AB725" t="inlineStr">
+      <c r="AB725" s="4" t="inlineStr">
         <is>
           <t>Waiting for Bri's reply on how to get WCEOB</t>
         </is>
@@ -68158,7 +68167,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J735" t="inlineStr">
+      <c r="J735" s="3" t="inlineStr">
         <is>
           <t>Finalized</t>
         </is>
@@ -68216,7 +68225,7 @@
       <c r="AA735" t="n">
         <v>78</v>
       </c>
-      <c r="AB735" t="inlineStr">
+      <c r="AB735" s="4" t="inlineStr">
         <is>
           <t>No auth on file - Adjusted</t>
         </is>
@@ -68970,7 +68979,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J744" t="inlineStr">
+      <c r="J744" s="3" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
@@ -69023,7 +69032,7 @@
       <c r="AA744" t="n">
         <v>80</v>
       </c>
-      <c r="AB744" t="inlineStr">
+      <c r="AB744" s="4" t="inlineStr">
         <is>
           <t>Corrected service line 1 to 99492, and resubmitted - Processed date 06/16/2026</t>
         </is>
@@ -69068,7 +69077,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J745" t="inlineStr">
+      <c r="J745" s="3" t="inlineStr">
         <is>
           <t>Rejected</t>
         </is>
@@ -69121,7 +69130,7 @@
       <c r="AA745" t="n">
         <v>80</v>
       </c>
-      <c r="AB745" t="inlineStr">
+      <c r="AB745" s="4" t="inlineStr">
         <is>
           <t>Corrected service line 1 to 99492, and resubmitted - Processed date 06/16/2026</t>
         </is>
@@ -69166,7 +69175,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J746" t="inlineStr">
+      <c r="J746" s="3" t="inlineStr">
         <is>
           <t>Denied</t>
         </is>
@@ -69214,7 +69223,7 @@
       <c r="AA746" t="n">
         <v>79</v>
       </c>
-      <c r="AB746" t="inlineStr">
+      <c r="AB746" s="4" t="inlineStr">
         <is>
           <t>Checking with biller</t>
         </is>
@@ -69259,7 +69268,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J747" t="inlineStr">
+      <c r="J747" s="3" t="inlineStr">
         <is>
           <t>Denied</t>
         </is>
@@ -69307,7 +69316,7 @@
       <c r="AA747" t="n">
         <v>79</v>
       </c>
-      <c r="AB747" t="inlineStr">
+      <c r="AB747" s="4" t="inlineStr">
         <is>
           <t>Checking with biller</t>
         </is>
@@ -74460,7 +74469,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J804" t="inlineStr">
+      <c r="J804" s="3" t="inlineStr">
         <is>
           <t>Denied</t>
         </is>
@@ -74518,7 +74527,7 @@
       <c r="AA804" t="n">
         <v>82</v>
       </c>
-      <c r="AB804" t="inlineStr">
+      <c r="AB804" s="4" t="inlineStr">
         <is>
           <t>Removed rendering, added servicing, changed from professional to DME, and resubmitted - Denied due to missing auth - I see rendering OON -  Processed date 06/12/2026</t>
         </is>
@@ -74827,7 +74836,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J808" t="inlineStr">
+      <c r="J808" s="3" t="inlineStr">
         <is>
           <t>Finalized</t>
         </is>
@@ -74885,7 +74894,7 @@
       <c r="AA808" t="n">
         <v>85</v>
       </c>
-      <c r="AB808" t="inlineStr">
+      <c r="AB808" s="4" t="inlineStr">
         <is>
           <t>Auth only included 63650 - Adjusted 63685</t>
         </is>
@@ -76313,7 +76322,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J825" t="inlineStr">
+      <c r="J825" s="3" t="inlineStr">
         <is>
           <t>Denied</t>
         </is>
@@ -76376,7 +76385,7 @@
       <c r="AA825" t="n">
         <v>58</v>
       </c>
-      <c r="AB825" t="inlineStr">
+      <c r="AB825" s="4" t="inlineStr">
         <is>
           <t>Delete 93923 that's bundling, and resubmitted -  93923 billed on claim 568263929 - Processed Date 06/25/2026</t>
         </is>
@@ -76421,7 +76430,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J826" t="inlineStr">
+      <c r="J826" s="3" t="inlineStr">
         <is>
           <t>Denied</t>
         </is>
@@ -76484,7 +76493,7 @@
       <c r="AA826" t="n">
         <v>58</v>
       </c>
-      <c r="AB826" t="inlineStr">
+      <c r="AB826" s="4" t="inlineStr">
         <is>
           <t>Delete 93923 that's bundling, and resubmitted -  93923 billed on claim 568263929 - Processed Date 06/25/2026</t>
         </is>
@@ -76529,7 +76538,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J827" t="inlineStr">
+      <c r="J827" s="3" t="inlineStr">
         <is>
           <t>Denied</t>
         </is>
@@ -76592,7 +76601,7 @@
       <c r="AA827" t="n">
         <v>58</v>
       </c>
-      <c r="AB827" t="inlineStr">
+      <c r="AB827" s="4" t="inlineStr">
         <is>
           <t>Delete 93923 that's bundling, and resubmitted -  93923 billed on claim 568263929 - Processed Date 06/25/2026</t>
         </is>
@@ -79996,7 +80005,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J866" t="inlineStr">
+      <c r="J866" s="3" t="inlineStr">
         <is>
           <t>PAID</t>
         </is>
@@ -80039,7 +80048,7 @@
       <c r="AA866" t="n">
         <v>52</v>
       </c>
-      <c r="AB866" t="inlineStr">
+      <c r="AB866" s="4" t="inlineStr">
         <is>
           <t>Pending posting</t>
         </is>
@@ -80084,7 +80093,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J867" t="inlineStr">
+      <c r="J867" s="3" t="inlineStr">
         <is>
           <t>PAID</t>
         </is>
@@ -80127,7 +80136,7 @@
       <c r="AA867" t="n">
         <v>52</v>
       </c>
-      <c r="AB867" t="inlineStr">
+      <c r="AB867" s="4" t="inlineStr">
         <is>
           <t>Pending posting</t>
         </is>
@@ -80436,7 +80445,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J871" t="inlineStr">
+      <c r="J871" s="3" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -80479,7 +80488,7 @@
       <c r="AA871" t="n">
         <v>86</v>
       </c>
-      <c r="AB871" t="inlineStr">
+      <c r="AB871" s="4" t="inlineStr">
         <is>
           <t>Uploaded MR - PIQ-88903761</t>
         </is>
@@ -81268,7 +81277,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J880" t="inlineStr">
+      <c r="J880" s="3" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -81311,7 +81320,7 @@
       <c r="AA880" t="n">
         <v>86</v>
       </c>
-      <c r="AB880" t="inlineStr">
+      <c r="AB880" s="4" t="inlineStr">
         <is>
           <t>Uploaded MR - PIQ-88903761</t>
         </is>
@@ -82151,7 +82160,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J891" t="inlineStr">
+      <c r="J891" s="3" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -82194,7 +82203,7 @@
       <c r="AA891" t="n">
         <v>78</v>
       </c>
-      <c r="AB891" t="inlineStr">
+      <c r="AB891" s="4" t="inlineStr">
         <is>
           <t>Uploaded MR - PIQ-88958247</t>
         </is>
@@ -86387,7 +86396,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J938" t="inlineStr">
+      <c r="J938" s="3" t="inlineStr">
         <is>
           <t>Finalized</t>
         </is>
@@ -86435,7 +86444,7 @@
       <c r="AA938" t="n">
         <v>88</v>
       </c>
-      <c r="AB938" t="inlineStr">
+      <c r="AB938" s="4" t="inlineStr">
         <is>
           <t>PR amount assigned as per EOB and adjusted</t>
         </is>
@@ -86480,7 +86489,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J939" t="inlineStr">
+      <c r="J939" s="3" t="inlineStr">
         <is>
           <t>Finalized</t>
         </is>
@@ -86528,7 +86537,7 @@
       <c r="AA939" t="n">
         <v>88</v>
       </c>
-      <c r="AB939" t="inlineStr">
+      <c r="AB939" s="4" t="inlineStr">
         <is>
           <t>PR amount assigned as per EOB and adjusted</t>
         </is>
@@ -92990,7 +92999,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J1014" t="inlineStr">
+      <c r="J1014" s="3" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -93033,7 +93042,7 @@
       <c r="AA1014" t="n">
         <v>78</v>
       </c>
-      <c r="AB1014" t="inlineStr">
+      <c r="AB1014" s="4" t="inlineStr">
         <is>
           <t>Uploaded MR - PIQ-88958247</t>
         </is>
@@ -98376,7 +98385,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J1076" t="inlineStr">
+      <c r="J1076" s="3" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -98419,7 +98428,7 @@
       <c r="AA1076" t="n">
         <v>86</v>
       </c>
-      <c r="AB1076" t="inlineStr">
+      <c r="AB1076" s="4" t="inlineStr">
         <is>
           <t>Uploaded MR - PIQ-88903858</t>
         </is>
@@ -98464,7 +98473,7 @@
           <t>No Payer</t>
         </is>
       </c>
-      <c r="J1077" t="inlineStr">
+      <c r="J1077" s="3" t="inlineStr">
         <is>
           <t>Pending</t>
         </is>
@@ -98507,7 +98516,7 @@
       <c r="AA1077" t="n">
         <v>86</v>
       </c>
-      <c r="AB1077" t="inlineStr">
+      <c r="AB1077" s="4" t="inlineStr">
         <is>
           <t>Uploaded MR - PIQ-88903858</t>
         </is>

</xml_diff>